<commit_message>
Add a data-entry copy of the cost sheet, without the commission column
The share is a term between two parties, not a product attribute, and the
people typing in a fifty-product catalogue are not the people who agreed it.
The importer already treats a missing column as "inherit the shop rate", so
the two files import identically apart from that one field - now covered by a
test that also asserts nothing reaches the commission log, since a log entry
claiming a rate was set would record a decision nobody made.

Both sheets gain a dropdown on the category column. Free text there drifts -
"protein" and "proteins" become two categories - and with several people
filling in different files it drifts on the first day.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/فایل-محصولات-SUPPEX.xlsx
+++ b/فایل-محصولات-SUPPEX.xlsx
@@ -500,7 +500,7 @@
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
@@ -3594,15 +3594,18 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:O1"/>
-  <dataValidations count="3">
+  <dataValidations count="4">
     <dataValidation sqref="K2:K400" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="فقط «بله» یا «خیر»" type="list">
       <formula1>"بله,خیر"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D2:D400" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="از لیست انتخاب کنید. دسته تازه لازم دارید؟ به ما بگویید." type="list">
+      <formula1>"پروتئین,کراتین,افزایش وزن,قبل تمرین,آمینو و BCAA,ویتامین و مکمل"</formula1>
     </dataValidation>
     <dataValidation sqref="J2:J400" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="درصد باید بین ۰ تا ۱۰۰ باشد. خالی یعنی درصد پیش‌فرض فروشگاه." type="decimal" operator="between">
       <formula1>0</formula1>
       <formula2>100</formula2>
     </dataValidation>
-    <dataValidation sqref="F2:F400" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="قیمت خرید به درهم است، نه تومان. مثلاً ۴۰" type="decimal" operator="between">
+    <dataValidation sqref="F2:F400" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="قیمت خرید به درهم است، نه تومان. مثلاً 40" type="decimal" operator="between">
       <formula1>0.01</formula1>
       <formula2>20000</formula2>
     </dataValidation>
@@ -3617,7 +3620,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3636,19 +3639,19 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="46" customHeight="1">
+    <row r="2" ht="50" customHeight="1">
       <c r="A2" s="10" t="inlineStr">
         <is>
-          <t>قانون اصلی</t>
+          <t>مهم‌ترین قانون</t>
         </is>
       </c>
       <c r="B2" s="11" t="inlineStr">
         <is>
-          <t>برای هر اندازه، یک سطر جداگانه. قوطی ۹۰۰ گرمی و ۲۲۷۰ گرمی دو خرید جدا با دو قیمت جدا هستند. نام فارسی را دقیقاً یکسان بنویسید؛ سیستم از روی همین نام، سطرها را یک محصول می‌کند.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="46" customHeight="1">
+          <t>برای هر اندازه، یک سطر جداگانه. قوطی ۹۰۰ گرمی و ۲۲۷۰ گرمی دو خرید جدا با دو قیمت جدا هستند. نام فارسی را در هر دو سطر دقیقاً یکسان بنویسید — سیستم از روی همین نام، سطرها را یک محصول می‌کند.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="50" customHeight="1">
       <c r="A3" s="10" t="inlineStr">
         <is>
           <t>محصول تک‌اندازه</t>
@@ -3660,7 +3663,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="46" customHeight="1">
+    <row r="4" ht="50" customHeight="1">
       <c r="A4" s="10" t="inlineStr">
         <is>
           <t>قیمت خرید (درهم)</t>
@@ -3668,11 +3671,11 @@
       </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
-          <t>عدد درهمی که برای خرید همان قوطی داده‌اید — مثلاً 40. تومان ننویسید. اگر قلمی را به تومان می‌خرید، این را خالی بگذارید و فقط «قیمت فروش» را پر کنید.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="46" customHeight="1">
+          <t>عدد درهمی که برای خرید همان یک قوطی داده‌اید — مثلاً 40. قیمت کارتن ننویسید. تومان هم ننویسید. اگر قلمی را به تومان می‌خرید، این را خالی بگذارید و فقط «قیمت فروش» را پر کنید.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="50" customHeight="1">
       <c r="A5" s="10" t="inlineStr">
         <is>
           <t>سود (تومان)</t>
@@ -3680,11 +3683,11 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>سودی که روی همان قوطی می‌خواهید. قیمت فروش خودکار از (درهم × نرخ روز) + سود ساخته می‌شود و با تغییر نرخ درهم خودش به‌روز می‌شود.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="46" customHeight="1">
+          <t>سودی که روی همان یک قوطی می‌خواهید. قیمت فروش خودکار از (درهم × نرخ روز) + سود ساخته می‌شود و با بالا و پایین شدن نرخ درهم، خودش به‌روز می‌شود.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="50" customHeight="1">
       <c r="A6" s="10" t="inlineStr">
         <is>
           <t>قیمت فروش (تومان)</t>
@@ -3696,7 +3699,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="46" customHeight="1">
+    <row r="7" ht="50" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
         <is>
           <t>تخفیف (تومان)</t>
@@ -3704,11 +3707,11 @@
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>مقداری که از قیمت کم می‌شود، نه قیمت دوم. بیشتر از نیمی از سود پذیرفته نمی‌شود.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="46" customHeight="1">
+          <t>مقداری که از قیمت کم می‌شود، نه قیمت دوم. بیشتر از نیمی از سود پذیرفته نمی‌شود. ندارید ← خالی.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="50" customHeight="1">
       <c r="A8" s="10" t="inlineStr">
         <is>
           <t>درصد همکاری</t>
@@ -3716,79 +3719,115 @@
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>خالی = درصد پیش‌فرض فروشگاه. فقط برای قلمی عدد بنویسید که جداگانه توافق شده — مثلاً قلمی که رقیب زیاد دارد. صفر یعنی «روی این قلم سهمی برداشته نشود» و با خالی یکی نیست.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="46" customHeight="1">
+          <t>خالی = درصد پیش‌فرض فروشگاه. فقط برای قلمی عدد بنویسید که جداگانه توافق شده — مثلاً قلمی که رقیب زیاد دارد و حاشیه سودش کم است. صفر یعنی «روی این قلم سهمی برداشته نشود» و با خالی یکی نیست.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="50" customHeight="1">
       <c r="A9" s="10" t="inlineStr">
         <is>
+          <t>دسته</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>از لیست کشویی همین ستون انتخاب کنید. دستی ننویسید — «پروتئین» و «پروتئین‌ها» دو دسته جدا می‌شوند. اگر دسته‌ای کم است، به ما بگویید تا اضافه کنیم.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="50" customHeight="1">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
           <t>طعم‌ها</t>
         </is>
       </c>
-      <c r="B9" s="11" t="inlineStr">
-        <is>
-          <t>با ویرگول جدا کنید: شکلاتی، وانیلی، توت فرنگی. یک‌بار برای هر محصول کافی است.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="46" customHeight="1">
-      <c r="A10" s="10" t="inlineStr">
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>با ویرگول جدا کنید: شکلاتی، وانیلی، توت فرنگی. فقط روی سطر اول هر محصول کافی است.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="50" customHeight="1">
+      <c r="A11" s="10" t="inlineStr">
         <is>
           <t>موجود</t>
         </is>
       </c>
-      <c r="B10" s="11" t="inlineStr">
+      <c r="B11" s="11" t="inlineStr">
         <is>
           <t>«بله» یا «خیر». خالی یعنی موجود.</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="46" customHeight="1">
-      <c r="A11" s="10" t="inlineStr">
+    <row r="12" ht="50" customHeight="1">
+      <c r="A12" s="10" t="inlineStr">
         <is>
           <t>تعداد وعده</t>
         </is>
       </c>
-      <c r="B11" s="11" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>چند وعده داخل همان قوطی است. اختیاری.</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="46" customHeight="1">
-      <c r="A12" s="10" t="inlineStr">
+    <row r="13" ht="50" customHeight="1">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>توضیح کوتاه</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>یک خط، زیر نام محصول در لیست دیده می‌شود.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="50" customHeight="1">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>توضیح کامل</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>متن کامل صفحه محصول. اختیاری — بعداً هم می‌شود نوشت.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="50" customHeight="1">
+      <c r="A15" s="10" t="inlineStr">
         <is>
           <t>عکس محصول</t>
         </is>
       </c>
-      <c r="B12" s="11" t="inlineStr">
-        <is>
-          <t>از این فایل خوانده نمی‌شود. بعد از ورود محصولات، از صفحه هر محصول در پنل آپلود می‌شود.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="46" customHeight="1">
-      <c r="A13" s="10" t="inlineStr">
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>داخل این فایل نمی‌آید. عکس‌ها را جداگانه بفرستید؛ نام فایل هر عکس را همان نام فارسی محصول بگذارید.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="50" customHeight="1">
+      <c r="A16" s="10" t="inlineStr">
         <is>
           <t>وقتی تمام شد</t>
         </is>
       </c>
-      <c r="B13" s="11" t="inlineStr">
-        <is>
-          <t>سطرهای نمونه (خاکستری) را پاک کنید، سپس File ← Save As ← CSV UTF-8 و همان فایل را در پنل، بخش «ورود گروهی محصولات» بارگذاری کنید. قبل از ثبت، پیش‌نمایش را نشانتان می‌دهد.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="46" customHeight="1">
-      <c r="A14" s="10" t="inlineStr">
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>سطرهای نمونه (خاکستری) را پاک کنید و همین فایل اکسل را پس بفرستید. لازم نیست تبدیلش کنید.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="50" customHeight="1">
+      <c r="A17" s="10" t="inlineStr">
         <is>
           <t>عنوان ستون‌ها</t>
         </is>
       </c>
-      <c r="B14" s="11" t="inlineStr">
-        <is>
-          <t>عوض نکنید و پاک نکنید. جابه‌جا کردن ستون‌ها اشکالی ندارد؛ سیستم از روی عنوان می‌خواند، نه جای ستون.</t>
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>عوض نکنید و پاک نکنید. ستون تازه هم اضافه نکنید.</t>
         </is>
       </c>
     </row>

</xml_diff>